<commit_message>
fix: map and pass VatBreakdownItem details on single-receipt load to edit form in both frontend and backend
</commit_message>
<xml_diff>
--- a/backend/ReceiptOCR.API/Data/fis_raporu_edit.xlsx
+++ b/backend/ReceiptOCR.API/Data/fis_raporu_edit.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Fiş_Tarihi</t>
   </si>
@@ -38,25 +38,19 @@
     <t>Toplam_Fiyat</t>
   </si>
   <si>
-    <t>2026-06-02</t>
-  </si>
-  <si>
-    <t>NIPA ELEKTRIK OTOMOSYO VE TIC LTD STI</t>
-  </si>
-  <si>
-    <t>6311361187</t>
-  </si>
-  <si>
-    <t>34</t>
+    <t>2026-06-18</t>
+  </si>
+  <si>
+    <t>CAGRI MAGAZACILIK A.S.</t>
+  </si>
+  <si>
+    <t>2200621779</t>
+  </si>
+  <si>
+    <t>00102</t>
   </si>
   <si>
     <t>2026-04-18</t>
-  </si>
-  <si>
-    <t>CAGRI MAGAZACILIK A.S.</t>
-  </si>
-  <si>
-    <t>2200621779</t>
   </si>
   <si>
     <t>00065</t>
@@ -136,11 +130,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName=""/>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.7694673538208" customWidth="1"/>
-    <col min="2" max="2" width="37.50625228881836" customWidth="1"/>
+    <col min="2" max="2" width="26.29755210876465" customWidth="1"/>
     <col min="3" max="3" width="11.634980201721191" customWidth="1"/>
     <col min="4" max="4" width="22.571548461914062" customWidth="1"/>
     <col min="5" max="5" width="10.570992469787598" customWidth="1"/>
@@ -189,42 +183,42 @@
         <v>11</v>
       </c>
       <c r="E2" s="0">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="F2" s="0">
-        <v>666.67</v>
+        <v>3044.52</v>
       </c>
       <c r="G2" s="0">
-        <v>133.33</v>
+        <v>30.45</v>
       </c>
       <c r="H2" s="0">
-        <v>800</v>
+        <v>3074.97</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E3" s="0">
         <v>20</v>
       </c>
       <c r="F3" s="0">
-        <v>190.71</v>
+        <v>519.04</v>
       </c>
       <c r="G3" s="0">
-        <v>38.14</v>
+        <v>103.81</v>
       </c>
       <c r="H3" s="0">
-        <v>228.85</v>
+        <v>622.85</v>
       </c>
     </row>
     <row r="4">
@@ -232,102 +226,128 @@
         <v>12</v>
       </c>
       <c r="B4" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="E4" s="0">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="F4" s="0">
-        <v>724.71</v>
+        <v>190.71</v>
       </c>
       <c r="G4" s="0">
-        <v>7.25</v>
+        <v>38.14</v>
       </c>
       <c r="H4" s="0">
-        <v>731.96</v>
+        <v>228.85</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="E5" s="0">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="F5" s="0">
-        <v>184.17</v>
+        <v>724.71</v>
       </c>
       <c r="G5" s="0">
-        <v>36.83</v>
+        <v>7.25</v>
       </c>
       <c r="H5" s="0">
-        <v>221</v>
+        <v>731.96</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E6" s="0">
         <v>20</v>
       </c>
       <c r="F6" s="0">
-        <v>225.25</v>
+        <v>184.17</v>
       </c>
       <c r="G6" s="0">
-        <v>45.03</v>
+        <v>36.83</v>
       </c>
       <c r="H6" s="0">
-        <v>270.28</v>
+        <v>221</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B7" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>23</v>
-      </c>
       <c r="E7" s="0">
+        <v>20</v>
+      </c>
+      <c r="F7" s="0">
+        <v>225.25</v>
+      </c>
+      <c r="G7" s="0">
+        <v>45.03</v>
+      </c>
+      <c r="H7" s="0">
+        <v>270.28</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="0">
         <v>1</v>
       </c>
-      <c r="F7" s="0">
+      <c r="F8" s="0">
         <v>157.17</v>
       </c>
-      <c r="G7" s="0">
+      <c r="G8" s="0">
         <v>1.57</v>
       </c>
-      <c r="H7" s="0">
+      <c r="H8" s="0">
         <v>158.74</v>
       </c>
     </row>

</xml_diff>